<commit_message>
Lambda 2023-11-21 oms  速卖通 sdk添加
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-plm/src/main/resources/excel/productLogistics.xlsx
+++ b/erp-server/erp-server-plm/src/main/resources/excel/productLogistics.xlsx
@@ -113,10 +113,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{.ena}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>{.propertyName}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -278,6 +274,10 @@
   </si>
   <si>
     <t>{.logisticsPropertyName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.ean}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -694,34 +694,34 @@
         <v>21</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O1" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="P1" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="S1" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="T1" s="2" t="s">
         <v>4</v>
@@ -730,10 +730,10 @@
         <v>13</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X1" s="3" t="s">
         <v>12</v>
@@ -742,25 +742,25 @@
         <v>5</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AB1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="AC1" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="AD1" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AE1" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AG1" s="2"/>
     </row>
@@ -781,85 +781,85 @@
         <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="K2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="P2" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="Q2" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R2" s="1" t="s">
         <v>10</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="U2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="V2" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="W2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="X2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="Z2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AA2" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="AB2" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AD2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>